<commit_message>
Learning Selenium from Mac
</commit_message>
<xml_diff>
--- a/Excel/caldata.xlsx
+++ b/Excel/caldata.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11114"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Learning\LearningSelenium\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/salimkhan/IdeaProjects/seleniumwebdriver/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F9A51D3-6E5A-4135-82CB-832C0FDD2381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B40A2F87-51FB-5441-B59C-8B5D7B55F932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33480" yWindow="1545" windowWidth="14400" windowHeight="7275" xr2:uid="{71CFE8B8-8ADB-C744-ADDA-33CB337DED60}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{71CFE8B8-8ADB-C744-ADDA-33CB337DED60}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
   <si>
     <t>Principal</t>
   </si>
@@ -59,9 +57,6 @@
     <t>month(s)</t>
   </si>
   <si>
-    <t>days(s)</t>
-  </si>
-  <si>
     <t>Simple Interest</t>
   </si>
   <si>
@@ -75,12 +70,22 @@
   </si>
   <si>
     <t>Fail</t>
+  </si>
+  <si>
+    <t>day(s)</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Failed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -90,12 +95,32 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="10"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -110,12 +135,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -134,9 +163,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -174,7 +203,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -280,7 +309,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -422,7 +451,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -431,130 +460,139 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B89EA7-F7CF-AD48-B9D7-A62DEC40E1B7}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="13.58203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.5"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.6640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.1640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="0">
+        <v>20000</v>
+      </c>
+      <c r="B2" s="0">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
-        <v>9</v>
+      <c r="C2" s="0">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1">
+        <v>24000</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s" s="3">
+        <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>20000</v>
-      </c>
-      <c r="B2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="0">
+        <v>30000</v>
+      </c>
+      <c r="B3" s="0">
+        <v>11</v>
+      </c>
+      <c r="C3" s="0">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F3" s="1">
+        <v>39900</v>
+      </c>
+      <c r="G3" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="H3" t="s" s="4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="0">
+        <v>40000</v>
+      </c>
+      <c r="B4" s="0">
+        <v>15</v>
+      </c>
+      <c r="C4" s="0">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1">
+        <v>42000</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="H4" t="s" s="5">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" s="0">
+        <v>50000</v>
+      </c>
+      <c r="B5" s="0">
+        <v>16</v>
+      </c>
+      <c r="C5" s="0">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="1">
-        <f>(A2*B2*C2)/100+A2</f>
-        <v>24000</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>30000</v>
-      </c>
-      <c r="B3">
-        <v>11</v>
-      </c>
-      <c r="C3">
-        <v>3</v>
-      </c>
-      <c r="D3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="1">
-        <f t="shared" ref="F3" si="0">(A3*B3*C3)/100+A3</f>
-        <v>39900</v>
-      </c>
-      <c r="G3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>40000</v>
-      </c>
-      <c r="B4">
-        <v>15</v>
-      </c>
-      <c r="C4">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="1">
-        <f>(A4*B4*C4)/1200+A4</f>
-        <v>42000</v>
-      </c>
-      <c r="G4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>50000</v>
-      </c>
-      <c r="B5">
-        <v>16</v>
-      </c>
-      <c r="C5">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="D5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s" s="0">
         <v>7</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
       </c>
       <c r="F5" s="1">
         <v>49000</v>
       </c>
-      <c r="G5" t="s">
-        <v>12</v>
+      <c r="G5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="H5" t="s" s="6">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>